<commit_message>
All sorts of odds and ends.
</commit_message>
<xml_diff>
--- a/TextConverter/src/main/resources/step.xlsx
+++ b/TextConverter/src/main/resources/step.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jamie\RemotelyBackedUp\Git\StepTextConversion\TextConverter\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FBE1D69-DE5A-4015-BEF4-17E05A4D1216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C403DA-50BC-4448-81EE-F7A68E34C4C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{6810EFB2-CF9F-4B19-9246-F88FA22FDC5D}"/>
   </bookViews>
@@ -629,9 +629,6 @@
     <t xml:space="preserve">             Mainly for use in the Sword config file, but may also appear on the STEPBible copyright page.</t>
   </si>
   <si>
-    <t xml:space="preserve">                                           Details of the organisation which holds the text.  Often this will be the same as the opwning organisation, in which case you can leave these entries blank.  But eg for DBL texts you will need details for DBL.</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">What it says on the tin.  You </t>
     </r>
@@ -740,6 +737,118 @@
     <t>This appears as the About parameter in Sword configuration files, and on the copyright page as the detailed copyright information.  Typically it gives copyright and permitted usage details (drawn from the fields above), but on some texts we go beyond this, for instance with background information about the translation.  It also includes acknowledgements and, on public modules, outline information about any changes we may have applied during processing.</t>
   </si>
   <si>
+    <t>#! Information to appear on the STEPBible Bible chooser.</t>
+  </si>
+  <si>
+    <t>Any copyright information or usage limitations from the text supplier.  On DBL texts it may be possible to pick this up from the metadata file, but you should check.  It is also worth looking on the websites of text suppliers to see if they supply more detailed information.
+You can either put all of the details into this one field, or you can split out various special parts of it into the fields above, in which case the system can apply standard formatting to it, to make it easier to read.
+If using multiple lines, don't forget to put backslash at the end of all but the last.</t>
+  </si>
+  <si>
+    <t>As stipulated by supplier.  Eg Can’t use more than 500 verses from one book.  This information ends up being used as part of the copyright statement.  If you give it here, I can format it neatly.  If that's not a great concern, you can simply include it as part of swordCopyrightStatement below.</t>
+  </si>
+  <si>
+    <t>As stipulated by supplier.  Eg Have to acknowledge.  This information ends up being used as part of the copyright statement.  If you give it here, I can format it neatly.  If that's not a great concern, you can simply include it as part of swordCopyrightStatement below.</t>
+  </si>
+  <si>
+    <t>Occasionally extended descriptive information is supplied by the text supplier, or we may want to add comments of our own.  This information ends up being used as part of the copyright statement.  If you give it here, I can format it neatly.  If that's not a great concern, you can simply include it as part of swordCopyrightStatement below.</t>
+  </si>
+  <si>
+    <t>#! Textual copyright information.</t>
+  </si>
+  <si>
+    <t>Describing the text</t>
+  </si>
+  <si>
+    <t>Normally processing starts from eg USX if available.  This says to start from existing OSIS.  Required only other inputs are available in addition to OSIS.</t>
+  </si>
+  <si>
+    <t>#! Other settings you may require.  They are used as-is, and therefore need to be complete configuration statements eg myParm#=123.</t>
+  </si>
+  <si>
+    <t>#! There must be only one statement per box.  You can add more rows if you need them, but make sure you copy %AdditionalStatements#= or %AdditionalIncludes#= to each.</t>
+  </si>
+  <si>
+    <t>Any 'include' or 'includeIfExists' statements.</t>
+  </si>
+  <si>
+    <t>#! Processing mechanics.  Also affected by the section marked 'CONTROL' above.</t>
+  </si>
+  <si>
+    <t>swordTypeOfDocument#=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                           Details of the organisation which holds the text.  Often this will be the same as the owning organisation, in which case you can leave these entries blank.  But eg for DBL texts you will need details for DBL.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>I don't police things here: I make the assumption that if you fail to supply a value which the spreadsheet describes as being required , it will be because you are going to include, from here, other textual config files which make good the deficit.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+The converter automatically defaults as many parameters as possible, including many of these defined here.  However, if you supply a non-blank value here, it will override the default.
+A strong yellow arrow with a copy icon below indicates that the lower item will normally be a direct copy of the earlier one, and need therefore be filled in only if you want to override that value.
+A semi-transparent yellow arrow with a copy icon and a 'calculate' icon indicates that the converter normally works out a value for itself, but will take the value at the start of the arrow if the calculation fails.  Fill in the field at the end of the arrow if you want to override this and force a value.
+A white arrow with a 'calculate' icon indicates that the lower element is normally deduced from the earlier one, but is not a direct copy of it.  As before, you can fill in the lower box to force your own value.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="13"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CAVEATS</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Some of the 'Calculated' fields organise for other elements to be assembled into what we have adopted as a 'standard' order.  If you override these by supplying your own value, you will need to ensure that value contains the information we normally require in these fields, and that it is ordered appropriately.  Regrettably as things stand you can determine what the content and order should be only by reference to the various configuration files in the Resources section of the converter JAR, or by reference to the code, particularly that in ConfigData.kt.
+Similarly in a number of cases, fields are described as being potentially derived from DBL data where available.  Again, if you wish to find out how they are derived, you will need to have recourse to the built-in configutation files and the code.  You should be aware that deriving information from DBL is, in any case, somewhat of a black art, in that the DBL metadata doesn't seem to be documented anywhere, and people therefore apply their own interpretation in deciding which fields should be used for what purpose.  And then at the end of all this, increasingly we are deciding to override that data anyway.
+All of this means that you may well need to do one or two runs and examine the outputs until you achieve what you want.</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -762,7 +871,29 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Fill in the cells below as appropriate.  They're colour-coded as follows:
+      <t xml:space="preserve">Fill in the cells below as appropriate.  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Column E indicates acceptable types of data or specific options in some cases.  If not specified, fields can contain free-form text.)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  Fields are colour-coded as follows:
 </t>
     </r>
     <r>
@@ -868,138 +999,6 @@
       <t>Optional.
    White:  These values are normally calculated but you can override them by providing your own values here if you wish (where there is no indication to the contrary).  In general, though, if it's white, you're unlikely to need to change it.</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Note that I do not police things here: I make the assumption that if you fail to supply a required value here, it may be because you are going to include, from here, other textual config files which make good the deficit.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-The processing automatically includes commonRoot.conf (from the converter JAR resources section), which supplies reasonable defaults for all parameters.  It then applies any non-blank definitions below.  Such definitions will override </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>all</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> other settings, and therefore will definitely be used.
-A strong yellow arrow with a copy icon below indicates that the lower item will normally be a direct copy of the earlier one, and need therefore be filled in only if you want to override that value.
-A semi-transparent yellow arrow with a copy icon and a 'calculate' icon indicates that the lower item may be defaulted by the system in a variety of ways, depending upon the circumstances – with the value from the upper box being used as a last resort.  Once again, you can enter a value here to force things.
-A white arrow with a 'calculate' icon indicates that the lower element is normally deduced from the earlier one, but is not a direct copy of it.  As before, you can fill in the lower box to force your own value.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="13"/>
-        <color rgb="FFFFFF00"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CAVEATS</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Some of the fields described as 'Calculated' rely upon quite complex calculations (calculations which, at present, I have decided are either too complicated to set out here, or are too liable to change).  You definitely can override these if you wish to, by giving values here, but bear in mind that the calculations may well be set up to organise things in a standard format which you may need to mimic.  Regrettably as things stand you can determine what that format is only by reference to the various configuration files in the Resources section of the converter JAR, or by reference to the code, particularly that in ConfigData.kt.
-Similarly in a number of cases, fields are described as being potentially derived from DBL data where available.  Again, if you wish to find out how they are derived, you will need to have recourse to the built-in configutation files and the code.  You should be aware that deriving information from DBL is, in any case, somewhat of a black art, in that the DBL metadata doesn't seem to be documented anywhere, and people therefore apply their own interpretation in deciding which fields should be used for what purpose.  And then at the end of all this, increasingly we are deciding to override that data anyway.
-All of this means that you may well need to do one or two runs and examine the outputs until you achieve what you want.</t>
-    </r>
-  </si>
-  <si>
-    <t>#! Information to appear on the STEPBible Bible chooser.</t>
-  </si>
-  <si>
-    <t>Any copyright information or usage limitations from the text supplier.  On DBL texts it may be possible to pick this up from the metadata file, but you should check.  It is also worth looking on the websites of text suppliers to see if they supply more detailed information.
-You can either put all of the details into this one field, or you can split out various special parts of it into the fields above, in which case the system can apply standard formatting to it, to make it easier to read.
-If using multiple lines, don't forget to put backslash at the end of all but the last.</t>
-  </si>
-  <si>
-    <t>As stipulated by supplier.  Eg Can’t use more than 500 verses from one book.  This information ends up being used as part of the copyright statement.  If you give it here, I can format it neatly.  If that's not a great concern, you can simply include it as part of swordCopyrightStatement below.</t>
-  </si>
-  <si>
-    <t>As stipulated by supplier.  Eg Have to acknowledge.  This information ends up being used as part of the copyright statement.  If you give it here, I can format it neatly.  If that's not a great concern, you can simply include it as part of swordCopyrightStatement below.</t>
-  </si>
-  <si>
-    <t>Occasionally extended descriptive information is supplied by the text supplier, or we may want to add comments of our own.  This information ends up being used as part of the copyright statement.  If you give it here, I can format it neatly.  If that's not a great concern, you can simply include it as part of swordCopyrightStatement below.</t>
-  </si>
-  <si>
-    <t>#! Textual copyright information.</t>
-  </si>
-  <si>
-    <t>Describing the text</t>
-  </si>
-  <si>
-    <t>Normally processing starts from eg USX if available.  This says to start from existing OSIS.  Required only other inputs are available in addition to OSIS.</t>
-  </si>
-  <si>
-    <t>#! Other settings you may require.  They are used as-is, and therefore need to be complete configuration statements eg myParm#=123.</t>
-  </si>
-  <si>
-    <t>#! There must be only one statement per box.  You can add more rows if you need them, but make sure you copy %AdditionalStatements#= or %AdditionalIncludes#= to each.</t>
-  </si>
-  <si>
-    <t>Any 'include' or 'includeIfExists' statements.</t>
-  </si>
-  <si>
-    <t>#! Processing mechanics.  Also affected by the section marked 'CONTROL' above.</t>
-  </si>
-  <si>
-    <t>swordTypeOfDocument#=</t>
   </si>
 </sst>
 </file>
@@ -5445,7 +5444,7 @@
   <sheetData>
     <row r="1" spans="1:7" s="57" customFormat="1" ht="192" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="67" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -5456,7 +5455,7 @@
     </row>
     <row r="2" spans="1:7" s="57" customFormat="1" ht="177.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="67" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B2" s="68"/>
       <c r="C2" s="68"/>
@@ -5467,7 +5466,7 @@
     </row>
     <row r="3" spans="1:7" s="57" customFormat="1" ht="168" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="70" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B3" s="68"/>
       <c r="C3" s="68"/>
@@ -6292,7 +6291,7 @@
         <v>118</v>
       </c>
       <c r="C78" s="61" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
       <c r="D78" s="60"/>
       <c r="E78" s="43"/>
@@ -6403,7 +6402,7 @@
         <v>2</v>
       </c>
       <c r="F88" s="16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G88" s="16"/>
     </row>
@@ -6427,7 +6426,7 @@
         <v>39</v>
       </c>
       <c r="F90" s="16" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G90" s="16"/>
     </row>
@@ -6543,7 +6542,7 @@
         <v>2</v>
       </c>
       <c r="F101" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G101" s="16"/>
     </row>
@@ -6614,7 +6613,7 @@
         <v>70</v>
       </c>
       <c r="F107" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G107" s="16"/>
     </row>
@@ -6631,14 +6630,14 @@
       <c r="A109" s="14"/>
       <c r="B109" s="18"/>
       <c r="C109" s="15" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D109" s="26"/>
       <c r="E109" s="17" t="s">
         <v>71</v>
       </c>
       <c r="F109" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G109" s="16"/>
     </row>
@@ -6686,7 +6685,7 @@
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="14"/>
       <c r="B114" s="33" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C114" s="34"/>
       <c r="D114" s="16"/>
@@ -6738,7 +6737,7 @@
         <v>2</v>
       </c>
       <c r="F118" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G118" s="16"/>
     </row>
@@ -6786,7 +6785,7 @@
         <v>2</v>
       </c>
       <c r="F122" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G122" s="16"/>
     </row>
@@ -6810,7 +6809,7 @@
         <v>2</v>
       </c>
       <c r="F124" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G124" s="16"/>
     </row>
@@ -6834,7 +6833,7 @@
         <v>2</v>
       </c>
       <c r="F126" s="16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G126" s="16"/>
     </row>
@@ -6850,10 +6849,10 @@
     <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="14"/>
       <c r="B129" s="33" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C129" s="66" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D129" s="16"/>
       <c r="E129" s="17"/>
@@ -6888,7 +6887,7 @@
         <v>2</v>
       </c>
       <c r="F132" s="48" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="G132" s="54"/>
     </row>
@@ -6912,7 +6911,7 @@
         <v>2</v>
       </c>
       <c r="F134" s="48" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="G134" s="16"/>
     </row>
@@ -6936,7 +6935,7 @@
         <v>2</v>
       </c>
       <c r="F136" s="48" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G136" s="16"/>
     </row>
@@ -6960,7 +6959,7 @@
         <v>2</v>
       </c>
       <c r="F138" s="48" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G138" s="16"/>
     </row>
@@ -7068,7 +7067,7 @@
         <v>2</v>
       </c>
       <c r="F148" s="48" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G148" s="16"/>
     </row>
@@ -7101,7 +7100,7 @@
     <row r="152" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="14"/>
       <c r="B152" s="33" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C152" s="34"/>
       <c r="D152" s="16"/>
@@ -7153,7 +7152,7 @@
         <v>51</v>
       </c>
       <c r="F156" s="16" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="G156" s="16"/>
     </row>
@@ -7177,7 +7176,7 @@
         <v>17</v>
       </c>
       <c r="F158" s="16" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G158" s="16"/>
     </row>
@@ -7198,10 +7197,10 @@
       </c>
       <c r="D160" s="19"/>
       <c r="E160" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F160" s="16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G160" s="16"/>
     </row>
@@ -7288,7 +7287,7 @@
     <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="14"/>
       <c r="B169" s="33" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C169" s="34"/>
       <c r="D169" s="16"/>
@@ -7299,7 +7298,7 @@
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="14"/>
       <c r="B170" s="33" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C170" s="34"/>
       <c r="D170" s="16"/>
@@ -7377,7 +7376,7 @@
         <v>2</v>
       </c>
       <c r="F176" s="16" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G176" s="16"/>
     </row>

</xml_diff>